<commit_message>
Update multiple Excel files with new data and analysis for club ranges, selector, clustered rounds, clutch score, golf recommendations, and strokes gained summary.
</commit_message>
<xml_diff>
--- a/club_ranges.xlsx
+++ b/club_ranges.xlsx
@@ -457,14 +457,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>42.36425000000003</v>
+        <v>42.496</v>
       </c>
       <c r="C2" t="n">
-        <v>84.23309999999995</v>
+        <v>83.41199999999998</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>42-84</t>
+          <t>42-83</t>
         </is>
       </c>
     </row>
@@ -475,14 +475,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84.45100000000008</v>
+        <v>81.83624999999995</v>
       </c>
       <c r="C3" t="n">
-        <v>114.0783999999999</v>
+        <v>109.8654000000001</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>84-114</t>
+          <t>81-109</t>
         </is>
       </c>
     </row>
@@ -493,14 +493,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>108.0975</v>
+        <v>106.2040000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>128.4039999999998</v>
+        <v>127.5999999999999</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>108-128</t>
+          <t>106-127</t>
         </is>
       </c>
     </row>
@@ -511,14 +511,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>130.5236</v>
+        <v>127.8786</v>
       </c>
       <c r="C5" t="n">
-        <v>144.776</v>
+        <v>142.8230999999999</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>130-144</t>
+          <t>127-142</t>
         </is>
       </c>
     </row>
@@ -529,14 +529,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>138.0354000000001</v>
+        <v>137.7482999999998</v>
       </c>
       <c r="C6" t="n">
-        <v>154.4812000000001</v>
+        <v>153.1431999999999</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>138-154</t>
+          <t>137-153</t>
         </is>
       </c>
     </row>
@@ -547,14 +547,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>151.29845</v>
+        <v>150.2533499999999</v>
       </c>
       <c r="C7" t="n">
-        <v>166.5779</v>
+        <v>165.37325</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>151-166</t>
+          <t>150-165</t>
         </is>
       </c>
     </row>
@@ -565,14 +565,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>161.4381999999998</v>
+        <v>161.3094</v>
       </c>
       <c r="C8" t="n">
-        <v>173.7279999999999</v>
+        <v>172.9973999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>161-173</t>
+          <t>161-172</t>
         </is>
       </c>
     </row>
@@ -583,14 +583,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>165.2879500000001</v>
+        <v>164.8889000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>181.9311000000002</v>
+        <v>182.4804000000002</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>165-181</t>
+          <t>164-182</t>
         </is>
       </c>
     </row>
@@ -601,14 +601,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>171.7995</v>
+        <v>171.8649000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>188.1008</v>
+        <v>187.8340000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>171-188</t>
+          <t>171-187</t>
         </is>
       </c>
     </row>
@@ -619,14 +619,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>179.207</v>
+        <v>179.7237499999999</v>
       </c>
       <c r="C11" t="n">
-        <v>213.1596000000001</v>
+        <v>212.5638</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>179-213</t>
+          <t>179-212</t>
         </is>
       </c>
     </row>
@@ -637,14 +637,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>202.4219999999997</v>
+        <v>201.4459999999997</v>
       </c>
       <c r="C12" t="n">
-        <v>231.4146</v>
+        <v>230.0788000000001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>202-231</t>
+          <t>201-230</t>
         </is>
       </c>
     </row>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>222.8079999999998</v>
+        <v>222.9420000000001</v>
       </c>
       <c r="C13" t="n">
-        <v>262.6869999999999</v>
+        <v>262.8849999999999</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Excel files with revised data for club ranges, club selector, clustered rounds, clutch score analysis, golf recommendations, and strokes gained summary. Enhance Golf Analytics notebook with updated cluster averages and scoring distribution analysis functions.
</commit_message>
<xml_diff>
--- a/club_ranges.xlsx
+++ b/club_ranges.xlsx
@@ -457,10 +457,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>42.496</v>
+        <v>42.40550000000003</v>
       </c>
       <c r="C2" t="n">
-        <v>83.41199999999998</v>
+        <v>83.63939999999995</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -475,14 +475,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81.83624999999995</v>
+        <v>78.85500000000008</v>
       </c>
       <c r="C3" t="n">
-        <v>109.8654000000001</v>
+        <v>100.492</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>81-109</t>
+          <t>78-100</t>
         </is>
       </c>
     </row>
@@ -493,14 +493,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>106.2040000000001</v>
+        <v>102.771</v>
       </c>
       <c r="C4" t="n">
-        <v>127.5999999999999</v>
+        <v>124.1584</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>106-127</t>
+          <t>102-124</t>
         </is>
       </c>
     </row>
@@ -511,14 +511,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>127.8786</v>
+        <v>121.8544999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>142.8230999999999</v>
+        <v>140.2331000000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>127-142</t>
+          <t>121-140</t>
         </is>
       </c>
     </row>
@@ -529,14 +529,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>137.7482999999998</v>
+        <v>135.6292499999998</v>
       </c>
       <c r="C6" t="n">
-        <v>153.1431999999999</v>
+        <v>149.8178000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>137-153</t>
+          <t>135-149</t>
         </is>
       </c>
     </row>
@@ -547,14 +547,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>150.2533499999999</v>
+        <v>150.5477999999998</v>
       </c>
       <c r="C7" t="n">
-        <v>165.37325</v>
+        <v>162.72065</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>150-165</t>
+          <t>150-162</t>
         </is>
       </c>
     </row>
@@ -565,14 +565,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>161.3094</v>
+        <v>159.0025999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>172.9973999999999</v>
+        <v>172.8574</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>161-172</t>
+          <t>159-172</t>
         </is>
       </c>
     </row>
@@ -583,14 +583,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>164.8889000000001</v>
+        <v>165.1000000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>182.4804000000002</v>
+        <v>182.1174000000002</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>164-182</t>
+          <t>165-182</t>
         </is>
       </c>
     </row>
@@ -601,14 +601,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>171.8649000000001</v>
+        <v>171.8997</v>
       </c>
       <c r="C10" t="n">
-        <v>187.8340000000001</v>
+        <v>188.0209</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>171-187</t>
+          <t>171-188</t>
         </is>
       </c>
     </row>
@@ -619,14 +619,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>179.7237499999999</v>
+        <v>180.5397499999999</v>
       </c>
       <c r="C11" t="n">
-        <v>212.5638</v>
+        <v>214.8974499999999</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>179-212</t>
+          <t>180-214</t>
         </is>
       </c>
     </row>
@@ -637,14 +637,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201.4459999999997</v>
+        <v>201.5219999999998</v>
       </c>
       <c r="C12" t="n">
-        <v>230.0788000000001</v>
+        <v>231.4766000000002</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>201-230</t>
+          <t>201-231</t>
         </is>
       </c>
     </row>
@@ -655,14 +655,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>222.9420000000001</v>
+        <v>222.1259999999998</v>
       </c>
       <c r="C13" t="n">
-        <v>262.8849999999999</v>
+        <v>263.1299999999998</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>222-262</t>
+          <t>222-263</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update multiple Excel files and Golf Analytics notebook with revised cluster averages, recommended clubs, and course data adjustments. Address deprecation warnings and enhance data consistency across analyses.
</commit_message>
<xml_diff>
--- a/club_ranges.xlsx
+++ b/club_ranges.xlsx
@@ -457,14 +457,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>42.40550000000003</v>
+        <v>43.3645</v>
       </c>
       <c r="C2" t="n">
-        <v>83.63939999999995</v>
+        <v>89.12169999999998</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>42-83</t>
+          <t>43-89</t>
         </is>
       </c>
     </row>
@@ -475,14 +475,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>78.85500000000008</v>
+        <v>79.26800000000004</v>
       </c>
       <c r="C3" t="n">
-        <v>100.492</v>
+        <v>100.764</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>78-100</t>
+          <t>79-100</t>
         </is>
       </c>
     </row>
@@ -493,14 +493,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>102.771</v>
+        <v>102.554</v>
       </c>
       <c r="C4" t="n">
-        <v>124.1584</v>
+        <v>123.3372000000001</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>102-124</t>
+          <t>102-123</t>
         </is>
       </c>
     </row>
@@ -511,14 +511,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>121.8544999999999</v>
+        <v>122.8123</v>
       </c>
       <c r="C5" t="n">
-        <v>140.2331000000001</v>
+        <v>139.0272000000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>121-140</t>
+          <t>122-139</t>
         </is>
       </c>
     </row>
@@ -529,14 +529,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>135.6292499999998</v>
+        <v>133.6712999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>149.8178000000001</v>
+        <v>149.7159999999998</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>135-149</t>
+          <t>133-149</t>
         </is>
       </c>
     </row>
@@ -547,14 +547,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>150.5477999999998</v>
+        <v>148.8272500000001</v>
       </c>
       <c r="C7" t="n">
-        <v>162.72065</v>
+        <v>161.3110000000001</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>150-162</t>
+          <t>148-161</t>
         </is>
       </c>
     </row>
@@ -565,14 +565,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>159.0025999999999</v>
+        <v>156.6791999999998</v>
       </c>
       <c r="C8" t="n">
-        <v>172.8574</v>
+        <v>173.4231</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>159-172</t>
+          <t>156-173</t>
         </is>
       </c>
     </row>
@@ -583,14 +583,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>165.1000000000001</v>
+        <v>164.0824</v>
       </c>
       <c r="C9" t="n">
-        <v>182.1174000000002</v>
+        <v>181.3310000000002</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>165-182</t>
+          <t>164-181</t>
         </is>
       </c>
     </row>
@@ -601,14 +601,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>171.8997</v>
+        <v>173.7672999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>188.0209</v>
+        <v>188.5556000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>171-188</t>
+          <t>173-188</t>
         </is>
       </c>
     </row>
@@ -619,14 +619,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>180.5397499999999</v>
+        <v>181.5264999999998</v>
       </c>
       <c r="C11" t="n">
-        <v>214.8974499999999</v>
+        <v>218.3850000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>180-214</t>
+          <t>181-218</t>
         </is>
       </c>
     </row>
@@ -637,14 +637,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201.5219999999998</v>
+        <v>205.0297499999998</v>
       </c>
       <c r="C12" t="n">
-        <v>231.4766000000002</v>
+        <v>232.64165</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>201-231</t>
+          <t>205-232</t>
         </is>
       </c>
     </row>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>222.1259999999998</v>
+        <v>222.0915000000001</v>
       </c>
       <c r="C13" t="n">
-        <v>263.1299999999998</v>
+        <v>263.7140000000005</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>

</xml_diff>